<commit_message>
changed input logic of clip model
</commit_message>
<xml_diff>
--- a/Models/CLIP/clip_trait_similarities_full_float.xlsx
+++ b/Models/CLIP/clip_trait_similarities_full_float.xlsx
@@ -413,1818 +413,3328 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B151"/>
+  <dimension ref="A1:D151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Trait</t>
+          <t>Negative Trait</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Probability</t>
+          <t>Negative Probability</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Positive Trait</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Positive Probability</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>a impractical person</t>
+          <t>a unlovable person</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.048171058297</t>
+          <t>0.000150074717</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>a modern person</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.026765683666</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>a simple person</t>
+          <t>a cruel person</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.032227523625</t>
+          <t>0.000336101599</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>a sweet person</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.002453613328</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>a confused person</t>
+          <t>a criminal person</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.031748224050</t>
+          <t>0.001912476844</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>a romantic person</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.001332696644</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>a unreflective person</t>
+          <t>a monstrous person</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.030709752813</t>
+          <t>0.000434878108</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>a youthful person</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.049511753023</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>a artificial person</t>
+          <t>a fraudulent person</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.025505160913</t>
+          <t>0.000279870525</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>a popular person</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.001276304480</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>a repressed person</t>
+          <t>a hateful person</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.024827096611</t>
+          <t>0.000529491692</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>a neat person</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.010831633583</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>a superficial person</t>
+          <t>a predatory person</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.023320853710</t>
+          <t>0.000461411750</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>a selfless person</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.000150607812</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>a unconvincing person</t>
+          <t>a dishonest person</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.022361282259</t>
+          <t>0.000392249174</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>a reflective person</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.004174063914</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>a shameless person</t>
+          <t>a malicious person</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0.022044518963</t>
+          <t>0.000816392479</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>a stylish person</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.267038434744</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>a pretentious person</t>
+          <t>a stupid person</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.021289356053</t>
+          <t>0.001198252314</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>a decisive person</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.000369496789</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>a one-dimensional person</t>
+          <t>a sadistic person</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.018955018371</t>
+          <t>0.000324350374</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>a open person</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.019544729963</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>a lazy person</t>
+          <t>a dirty person</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.017887335271</t>
+          <t>0.001249822089</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>a sane person</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0.000359039550</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>a unambitious person</t>
+          <t>a venomous person</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.016491476446</t>
+          <t>0.000225620824</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>a high-spirited person</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0.003481811378</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>a naive person</t>
+          <t>a barbaric person</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0.016361610964</t>
+          <t>0.000219747919</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>a protective person</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.000137329684</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>a troublesome person</t>
+          <t>a unlikeable person</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0.016333609819</t>
+          <t>0.001023149933</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>a sophisticated person</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.004011761863</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>a egocentric person</t>
+          <t>a deceitful person</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0.016049310565</t>
+          <t>0.000929815287</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>a hopeful person</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0.004723261576</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>a rowdy person</t>
+          <t>a neglectful person</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0.015839988366</t>
+          <t>0.000387263281</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>a dynamic person</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.005482936744</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>a oppressed person</t>
+          <t>a false person</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0.015666559339</t>
+          <t>0.000520657690</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>a elegant person</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.005257042591</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>a disorganised person</t>
+          <t>a disloyal person</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0.015361781232</t>
+          <t>0.000131520399</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>a freethinking person</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.006024148315</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>a vulnerable person</t>
+          <t>a heartless person</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0.015188256279</t>
+          <t>0.000162972952</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>a cultured person</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0.000846582174</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>a ridiculous person</t>
+          <t>a uncaring person</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0.013955883682</t>
+          <t>0.000466899743</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>a tasteful person</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0.005811794195</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>a disorderly person</t>
+          <t>a vindictive person</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.013698670082</t>
+          <t>0.000309516763</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>a responsive person</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0.001374494983</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>a absentminded person</t>
+          <t>a narcissistic person</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0.013357726857</t>
+          <t>0.000918248377</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>a forgiving person</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0.000070257622</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>a bland person</t>
+          <t>a ignorant person</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0.012891089544</t>
+          <t>0.000132854402</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>a flexible person</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0.000736941642</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>a short-sighted person</t>
+          <t>a unreliable person</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0.012640427798</t>
+          <t>0.000602584623</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>a progressive person</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0.001635503606</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>a scornful person</t>
+          <t>a ungrateful person</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0.011576764286</t>
+          <t>0.000084131643</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>a adventurous person</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0.001313790563</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>a unimaginative person</t>
+          <t>a treacherous person</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0.010724824853</t>
+          <t>0.000332902622</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>a sociable person</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0.001106875599</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>a coarse person</t>
+          <t>a disturbing person</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0.010686476715</t>
+          <t>0.001174034318</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>a amusing person</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>0.002462493023</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>a presumptuous person</t>
+          <t>a selfish person</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0.010384392925</t>
+          <t>0.000026744770</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>a principled person</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0.000409621745</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>a unimpressive person</t>
+          <t>a destructive person</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0.010226285085</t>
+          <t>0.000134242378</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>a strong-willed person</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0.002847908530</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>a charmless person</t>
+          <t>a inconsiderate person</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0.009968741797</t>
+          <t>0.000089813235</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>a energetic person</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0.016650792211</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>a unpolished person</t>
+          <t>a obnoxious person</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0.009597768076</t>
+          <t>0.001547082094</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>a tidy person</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0.006644611247</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>a criminal person</t>
+          <t>a disrespectful person</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0.009370841086</t>
+          <t>0.001128091244</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>a dignified person</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0.000930883514</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>a meddlesome person</t>
+          <t>a insincere person</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0.009272961877</t>
+          <t>0.000690404326</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>a cool person</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0.027366410941</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>a uncreative person</t>
+          <t>a desperate person</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0.009218875319</t>
+          <t>0.000443835248</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>a stable person</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0.001853508758</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>a erratic person</t>
+          <t>a deceptive person</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0.009107233025</t>
+          <t>0.000547057600</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>a precise person</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0.000885835849</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>a pompous person</t>
+          <t>a hostile person</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0.008931014687</t>
+          <t>0.000372237817</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>a personable person</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0.006779646501</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>a careless person</t>
+          <t>a grim person</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0.008211535402</t>
+          <t>0.000184456396</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>a alert person</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>0.005696808454</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>a uncooperative person</t>
+          <t>a unfriendly person</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0.007887307554</t>
+          <t>0.001351800165</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>a disciplined person</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0.000662010454</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>a obnoxious person</t>
+          <t>a unstable person</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0.007580478676</t>
+          <t>0.000495065993</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>a realistic person</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>0.000715615577</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>a graceless person</t>
+          <t>a irresponsible person</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0.007565859705</t>
+          <t>0.000547056610</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>a trusting person</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0.000040429528</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>a dismissive person</t>
+          <t>a cowardly person</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0.007313150913</t>
+          <t>0.000130539964</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>a gentle person</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>0.001116719330</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>a prejudiced person</t>
+          <t>a weak-willed person</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0.007311296184</t>
+          <t>0.000968159526</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>a tolerant person</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0.000221962386</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>a contradictory person</t>
+          <t>a shallow person</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0.007202944253</t>
+          <t>0.000789911544</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>a original person</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0.006588905118</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>a tactless person</t>
+          <t>a insulting person</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0.007164072711</t>
+          <t>0.000271772529</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>a active person</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0.009263921529</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>a disruptive person</t>
+          <t>a unprincipled person</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0.007101641037</t>
+          <t>0.000216535060</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>a mature person</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>0.001988513162</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>a unhealthy person</t>
+          <t>a prejudiced person</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0.007025761995</t>
+          <t>0.001492148265</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>a purposeful person</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>0.000903421082</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>a dull person</t>
+          <t>a narrow-minded person</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0.006934220903</t>
+          <t>0.000508789730</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>a gracious person</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0.002258995548</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>a unfriendly person</t>
+          <t>a perverse person</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0.006623649970</t>
+          <t>0.000794364081</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>a intuitive person</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>0.000179098002</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>a misguided person</t>
+          <t>a greedy person</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>0.006578324828</t>
+          <t>0.000192909749</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>a relaxed person</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>0.018229264766</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>a crude person</t>
+          <t>a weak person</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>0.006560331676</t>
+          <t>0.000374640309</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>a ambitious person</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>0.000976948533</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>a tasteless person</t>
+          <t>a thoughtless person</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>0.006441793405</t>
+          <t>0.000951542112</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>a secure person</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>0.000932824390</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>a abrupt person</t>
+          <t>a artificial person</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>0.006362543441</t>
+          <t>0.005205259193</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>a cooperative person</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>0.004875797313</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>a cold person</t>
+          <t>a unimpressive person</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0.006257059053</t>
+          <t>0.002087058732</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>a fun-loving person</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>0.005659941118</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>a fickle person</t>
+          <t>a aggressive person</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0.006137839518</t>
+          <t>0.000370708818</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>a captivating person</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>0.000723758363</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>a dirty person</t>
+          <t>a unappreciative person</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>0.006123935804</t>
+          <t>0.000143541401</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>a eloquent person</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>0.000366554887</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>a resentful person</t>
+          <t>a frightening person</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>0.005880463868</t>
+          <t>0.000485832395</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>a nice person</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>0.002700993558</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>a stupid person</t>
+          <t>a dull person</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0.005871262867</t>
+          <t>0.001415183651</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>a heroic person</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>0.001588113955</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>a disturbing person</t>
+          <t>a brutal person</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>0.005752597935</t>
+          <t>0.000843181973</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>a diligent person</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>0.001331670210</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>a disrespectful person</t>
+          <t>a sloppy person</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0.005527494475</t>
+          <t>0.000227105193</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>a peaceful person</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>0.005131513346</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>a gloomy person</t>
+          <t>a scheming person</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0.005210458301</t>
+          <t>0.000916998775</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>a charming person</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>0.004582520109</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>a neurotic person</t>
+          <t>a callous person</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0.005144963507</t>
+          <t>0.000494075532</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>a practical person</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0.003140710527</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>a remorseless person</t>
+          <t>a devious person</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0.005057224538</t>
+          <t>0.000626733468</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>a easy-going person</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>0.019123500213</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>a unlikeable person</t>
+          <t>a intolerant person</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0.005013276823</t>
+          <t>0.000225231284</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>a charismatic person</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>0.003737505060</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>a weak-willed person</t>
+          <t>a sly person</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>0.004743832629</t>
+          <t>0.000570459059</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>a exciting person</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>0.004254579544</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>a thoughtless person</t>
+          <t>a miserable person</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>0.004662373569</t>
+          <t>0.000858128071</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>a innovative person</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>0.000770760118</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>a easily discouraged person</t>
+          <t>a tasteless person</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>0.004659973551</t>
+          <t>0.001314683119</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>a humble person</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>0.002784065204</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>a irritable person</t>
+          <t>a remorseless person</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>0.004617874511</t>
+          <t>0.001032122993</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>a rational person</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>0.000654230418</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>a deceitful person</t>
+          <t>a discouraging person</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>0.004555942491</t>
+          <t>0.000412249035</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>a sharing person</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>0.000291854783</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>a narcissistic person</t>
+          <t>a lazy person</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>0.004499284085</t>
+          <t>0.003650584491</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>a insightful person</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>0.000499041169</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>a scheming person</t>
+          <t>a careless person</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>0.004493143875</t>
+          <t>0.001675876323</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>a observant person</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>0.000893556920</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>a insecure person</t>
+          <t>a uncooperative person</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>0.004450166598</t>
+          <t>0.001609708415</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>a perceptive person</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>0.000806338096</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>a uncharitable person</t>
+          <t>a insensitive person</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>0.004431937821</t>
+          <t>0.000162138924</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>a conscientious person</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>0.005271500908</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>a moody person</t>
+          <t>a irrational person</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>0.004403827246</t>
+          <t>0.000124469967</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>a optimistic person</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>0.002249158686</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>a miserable person</t>
+          <t>a morbid person</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0.004204670899</t>
+          <t>0.000639764301</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>a courteous person</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>0.000709702726</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>a brutal person</t>
+          <t>a paranoid person</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>0.004131469410</t>
+          <t>0.000188959631</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>a logical person</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>0.000261380017</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>a rigid person</t>
+          <t>a resentful person</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>0.004110341892</t>
+          <t>0.001200130209</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>a self-sufficient person</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>0.011703236029</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>a crass person</t>
+          <t>a pompous person</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>0.004102290608</t>
+          <t>0.001822706545</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>a imaginative person</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>0.000995518058</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>a unrealistic person</t>
+          <t>a foolish person</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>0.004029149655</t>
+          <t>0.000288397365</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>a calm person</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>0.001650388469</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>a malicious person</t>
+          <t>a scornful person</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>0.004000204615</t>
+          <t>0.002362688538</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>a engaging person</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>0.001502813306</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>a undisciplined person</t>
+          <t>a slow person</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>0.003926711623</t>
+          <t>0.000352191128</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>a witty person</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>0.000560558692</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>a perverse person</t>
+          <t>a cold person</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>0.003892268753</t>
+          <t>0.001276983763</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>a patient person</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>0.001198332408</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>a shallow person</t>
+          <t>a conceited person</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>0.003870429937</t>
+          <t>0.000476781890</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>a adaptable person</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>0.004484424368</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>a childish person</t>
+          <t>a one-dimensional person</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>0.003667449113</t>
+          <t>0.003868478118</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>a passionate person</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>0.000468336599</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>a aimless person</t>
+          <t>a tactless person</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>0.003639880335</t>
+          <t>0.001462096232</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>a clear-headed person</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>0.000666949491</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>a insincere person</t>
+          <t>a superficial person</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>0.003382887691</t>
+          <t>0.004759480711</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>a sympathetic person</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>0.000603341323</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>a morbid person</t>
+          <t>a unhealthy person</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>0.003134752158</t>
+          <t>0.001433871454</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>a well-read person</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>0.003606987419</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>a devious person</t>
+          <t>a undisciplined person</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>0.003070920706</t>
+          <t>0.000801391841</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>a self-reliant person</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>0.002701668534</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>a mistaken person</t>
+          <t>a uncharitable person</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>0.003014529590</t>
+          <t>0.000904496992</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>a affectionate person</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>0.000148646912</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>a unreliable person</t>
+          <t>a ridiculous person</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>0.002952583134</t>
+          <t>0.002848218195</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>a thorough person</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>0.000557779276</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>a sly person</t>
+          <t>a charmless person</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>0.002795177512</t>
+          <t>0.002034497214</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>a cheerful person</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>0.009532755241</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>a deceptive person</t>
+          <t>a gloomy person</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>0.002680497942</t>
+          <t>0.001063390286</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>a extraordinary person</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>0.000587240851</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>a irresponsible person</t>
+          <t>a bland person</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>0.002680482576</t>
+          <t>0.002630912466</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>a focused person</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>0.000696217467</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>a hateful person</t>
+          <t>a unimaginative person</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>0.002594432561</t>
+          <t>0.002188800136</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>a organised person</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>0.005664865952</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>a false person</t>
+          <t>a sneaky person</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>0.002551156795</t>
+          <t>0.000112532703</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>a empathetic person</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>0.000377990829</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>a narrow-minded person</t>
+          <t>a petty person</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>0.002492995933</t>
+          <t>0.000450485124</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>a confident person</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>0.011969235726</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>a unstable person</t>
+          <t>a neurotic person</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>0.002425746992</t>
+          <t>0.001050021616</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>a enthusiastic person</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>0.004418851342</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>a callous person</t>
+          <t>a crass person</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>0.002420889214</t>
+          <t>0.000837226864</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>a courageous person</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>0.000374610303</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>a frightening person</t>
+          <t>a stingy person</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>0.002380512888</t>
+          <t>0.000082016588</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>a fair person</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>0.001743989065</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>a conceited person</t>
+          <t>a disruptive person</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>0.002336162142</t>
+          <t>0.001449349103</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>a dedicated person</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>0.000252730591</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>a uncaring person</t>
+          <t>a oppressed person</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>0.002287736628</t>
+          <t>0.003197363578</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>a creative person</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>0.002344592474</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>a predatory person</t>
+          <t>a pretentious person</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>0.002260837937</t>
+          <t>0.004344928078</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>a impressive person</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>0.002574638231</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>a obsessive person</t>
+          <t>a gullible person</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>0.002212825464</t>
+          <t>0.000213965817</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>a articulate person</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>0.001047890750</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>a petty person</t>
+          <t>a crude person</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>0.002207315760</t>
+          <t>0.001338885399</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>a efficient person</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>0.004368177615</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>a desperate person</t>
+          <t>a graceless person</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>0.002174715977</t>
+          <t>0.001544092898</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>a appreciative person</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>0.000232919148</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>a abrasive person</t>
+          <t>a disorderly person</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>0.002145811915</t>
+          <t>0.002795713721</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>a resourceful person</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>0.002057489939</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>a monstrous person</t>
+          <t>a envious person</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>0.002130823443</t>
+          <t>0.000414513488</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>a healthy person</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>0.006594751496</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>a envious person</t>
+          <t>a repressed person</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>0.002031055978</t>
+          <t>0.005066914484</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>a independent person</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>0.002054842887</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>a discouraging person</t>
+          <t>a possessive person</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>0.002019956708</t>
+          <t>0.000065120730</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>a faithful person</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>0.000102704616</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>a dishonest person</t>
+          <t>a egocentric person</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>0.001921964111</t>
+          <t>0.003275478957</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>a attractive person</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>0.002182738623</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>a neglectful person</t>
+          <t>a troublesome person</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>0.001897526556</t>
+          <t>0.003333475906</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>a clean person</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>0.014027498662</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>a weak person</t>
+          <t>a abrasive person</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>0.001835672883</t>
+          <t>0.000437932933</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>a punctual person</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>0.002353472635</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>a hostile person</t>
+          <t>a meddlesome person</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>0.001823904458</t>
+          <t>0.001892500906</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>a admirable person</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>0.000496596214</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>a aggressive person</t>
+          <t>a impractical person</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>0.001816415926</t>
+          <t>0.009831137955</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>a educated person</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>0.001026474871</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>a slow person</t>
+          <t>a dismissive person</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>0.001725685550</t>
+          <t>0.001492521027</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>a strong person</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>0.000730750791</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>a cruel person</t>
+          <t>a misguided person</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>0.001646849094</t>
+          <t>0.001342549920</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>a lovely person</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>0.004936452955</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>a treacherous person</t>
+          <t>a fickle person</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>0.001631162246</t>
+          <t>0.001252657385</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>a capable person</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>0.000496615132</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>a sadistic person</t>
+          <t>a naive person</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>0.001589269727</t>
+          <t>0.003339190269</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>a open-minded person</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>0.000830082688</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>a vindictive person</t>
+          <t>a unconvincing person</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>0.001516572782</t>
+          <t>0.004563687835</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>a authentic person</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>0.002216545166</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>a foolish person</t>
+          <t>a amoral person</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>0.001413105289</t>
+          <t>0.000231909769</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>a honourable person</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>0.000059520968</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>a fraudulent person</t>
+          <t>a uncreative person</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>0.001371319755</t>
+          <t>0.001881447970</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>a determined person</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>0.004500980023</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>a insulting person</t>
+          <t>a aimless person</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>0.001331648440</t>
+          <t>0.000742856122</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>a generous person</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>0.000707714295</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>a amoral person</t>
+          <t>a coarse person</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>0.001136326347</t>
+          <t>0.002180982381</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>a interesting person</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>0.002513213083</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>a sloppy person</t>
+          <t>a unreflective person</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>0.001112784608</t>
+          <t>0.006267469376</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>a wise person</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>0.000333650794</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>a venomous person</t>
+          <t>a insecure person</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>0.001105511445</t>
+          <t>0.000908227579</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>a respectful person</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>0.001034089597</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>a intolerant person</t>
+          <t>a disorganised person</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>0.001103598508</t>
+          <t>0.003135168226</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>a good-natured person</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>0.018594231457</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>a barbaric person</t>
+          <t>a shameless person</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>0.001076739049</t>
+          <t>0.004498997238</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>a considerate person</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>0.000142458317</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>a unprincipled person</t>
+          <t>a difficult person</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>0.001060992479</t>
+          <t>0.000084332947</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>a warm person</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>0.008309924044</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>a gullible person</t>
+          <t>a unambitious person</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>0.001048401464</t>
+          <t>0.003365720157</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>a compassionate person</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>0.000211480306</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>a submissive person</t>
+          <t>a short-sighted person</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>0.000988991465</t>
+          <t>0.002579740481</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>a skillful person</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>0.001395724830</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>a greedy person</t>
+          <t>a erratic person</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>0.000945229840</t>
+          <t>0.001858666772</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>a thoughtful person</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>0.001119404216</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>a paranoid person</t>
+          <t>a obsessive person</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>0.000925874861</t>
+          <t>0.000451611268</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>a lovable person</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>0.000366976717</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>a grim person</t>
+          <t>a childish person</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>0.000903809618</t>
+          <t>0.000748482533</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>a responsible person</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>0.001228264766</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>a disobedient person</t>
+          <t>a irritable person</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>0.000898200320</t>
+          <t>0.000942449493</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>a caring person</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>0.000469656050</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>a heartless person</t>
+          <t>a absentminded person</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>0.000798543799</t>
+          <t>0.002726147650</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>a understanding person</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>0.000492246007</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>a insensitive person</t>
+          <t>a unpolished person</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>0.000794458727</t>
+          <t>0.001958793495</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>a smart person</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>0.002050657524</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>a unlovable person</t>
+          <t>a unrealistic person</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>0.000735345820</t>
+          <t>0.000822293456</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>a loving person</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>0.000634400698</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>a unappreciative person</t>
+          <t>a easily discouraged person</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>0.000703329337</t>
+          <t>0.000951044902</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>a approachable person</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>0.005415380467</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>a destructive person</t>
+          <t>a confused person</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>0.000657768163</t>
+          <t>0.006479421165</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>a clever person</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>0.000729500200</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>a ignorant person</t>
+          <t>a disobedient person</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>0.000650964794</t>
+          <t>0.000183311626</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>a knowledgeable person</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>0.000604084111</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>a disloyal person</t>
+          <t>a submissive person</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>0.000644430867</t>
+          <t>0.000201840958</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>a friendly person</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>0.003107514465</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>a cowardly person</t>
+          <t>a contradictory person</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>0.000639626931</t>
+          <t>0.001470029238</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>a brilliant person</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>0.001999275759</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>a irrational person</t>
+          <t>a presumptuous person</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>0.000609883631</t>
+          <t>0.002119318349</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>a loyal person</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>0.000102106933</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>a sneaky person</t>
+          <t>a rowdy person</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>0.000551393954</t>
+          <t>0.003232746385</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>a reliable person</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>0.000338250858</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>a inconsiderate person</t>
+          <t>a moody person</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>0.000440070144</t>
+          <t>0.000898765167</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>a hardworking person</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>0.003148135496</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>a difficult person</t>
+          <t>a abrupt person</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>0.000413219212</t>
+          <t>0.001298516756</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>a intelligent person</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>0.000404578546</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>a ungrateful person</t>
+          <t>a vulnerable person</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>0.000412232854</t>
+          <t>0.003099730238</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>a kind person</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>0.000672465074</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>a stingy person</t>
+          <t>a mistaken person</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>0.000401868660</t>
+          <t>0.000615223602</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>a genuine person</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>0.002339589410</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>a possessive person</t>
+          <t>a rigid person</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>0.000319083367</t>
+          <t>0.000838871638</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>a trustworthy person</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>0.000188271064</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>a selfish person</t>
+          <t>a simple person</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>0.000131045250</t>
+          <t>0.006577240303</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>a honest person</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>0.000717367569</t>
         </is>
       </c>
     </row>

</xml_diff>